<commit_message>
Power supply fix Draftsman added
</commit_message>
<xml_diff>
--- a/Project Outputs for EMT Rack Temperature Controller/Bill of Material/Rack Temperature & Fan Controller_BoM_Rev.1.0._2026-03-11.xlsx
+++ b/Project Outputs for EMT Rack Temperature Controller/Bill of Material/Rack Temperature & Fan Controller_BoM_Rev.1.0._2026-03-11.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Altium\Repositories\Temperature-Controller\Project Outputs for EMT Rack Temperature Controller\Bill of Material\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B90DC15D-41D5-410E-BA7D-9F059E960EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A62F1BE-735C-4CAE-B6F6-3FA48B9C7B12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{B859A70A-EAE8-42F1-88BB-3A3FA408F9D4}"/>
+    <workbookView xWindow="42450" yWindow="5535" windowWidth="28800" windowHeight="15345" xr2:uid="{839DB629-0655-494B-972E-75E570D7947C}"/>
   </bookViews>
   <sheets>
     <sheet name="Rack Temperature &amp; Fan Controll" sheetId="1" r:id="rId1"/>
@@ -68,7 +68,7 @@
     <t>Capacitor Non-Polar</t>
   </si>
   <si>
-    <t>C2, C5, C8</t>
+    <t>C1, C4, C8</t>
   </si>
   <si>
     <t>CAP-0805</t>
@@ -83,7 +83,7 @@
     <t>100nF</t>
   </si>
   <si>
-    <t>C3, C4, C7</t>
+    <t>C2, C3, C7</t>
   </si>
   <si>
     <t>82-13-46</t>
@@ -95,7 +95,7 @@
     <t>470uF 16V</t>
   </si>
   <si>
-    <t>C1, C6</t>
+    <t>C5, C6</t>
   </si>
   <si>
     <t>CAP-ELCO-SMD-FK1</t>
@@ -637,7 +637,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CEBB74B-E354-4579-83D2-1D67416378FD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60F17AF7-0521-4CE6-AB8E-6A7C804A26C5}">
   <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>